<commit_message>
docs y calibracion: actualizar planillas y notas de calibracion v4 e incorporar modulo de estructura para filtro
</commit_message>
<xml_diff>
--- a/02_Hito2_Instrumentacion_Sensores/02_Firmware_Test_Sensores/subhito2_2_v4/PLANILLA_CALIBRACION_ENSAYOS_2_Y_3.xlsx
+++ b/02_Hito2_Instrumentacion_Sensores/02_Firmware_Test_Sensores/subhito2_2_v4/PLANILLA_CALIBRACION_ENSAYOS_2_Y_3.xlsx
@@ -1,22 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/88ed92497b16fe2a/Documentos/ENZO/Domotica/SistemaUF/02_Hito2_Instrumentacion_Sensores/02_Firmware_Test_Sensores/subhito2_2_v4/EN_USO_firmware_planta/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\antigravity\Antigravity IDE\PROYECTOS\Tesis\Planta-Ultrafiltracion\02_Hito2_Instrumentacion_Sensores\02_Firmware_Test_Sensores\subhito2_2_v4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_D2AB47894A8A085B242471DB400DEFF5EDE26276" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="-105" windowWidth="19425" windowHeight="10425" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Ensayo 2 - Bomba (mL-rev)" sheetId="1" r:id="rId1"/>
     <sheet name="Ensayo 3 - Caudal Alimentacion" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -298,7 +297,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="7">
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
@@ -619,31 +618,15 @@
     <xf numFmtId="164" fontId="9" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -653,16 +636,32 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="168" fontId="11" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="169" fontId="11" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="168" fontId="11" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="170" fontId="11" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="11" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -705,6 +704,7 @@
           </a:p>
         </c:rich>
       </c:tx>
+      <c:layout/>
       <c:overlay val="1"/>
     </c:title>
     <c:autoTitleDeleted val="0"/>
@@ -779,28 +779,28 @@
                 <c:formatCode>0.0</c:formatCode>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>280</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>430</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>597</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>720</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
+                  <c:v>820</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0</c:v>
+                  <c:v>915</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0</c:v>
+                  <c:v>960</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0</c:v>
+                  <c:v>1080</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -847,6 +847,7 @@
               </a:p>
             </c:rich>
           </c:tx>
+          <c:layout/>
           <c:overlay val="1"/>
         </c:title>
         <c:numFmt formatCode="0.0" sourceLinked="1"/>
@@ -881,6 +882,7 @@
               </a:p>
             </c:rich>
           </c:tx>
+          <c:layout/>
           <c:overlay val="1"/>
         </c:title>
         <c:numFmt formatCode="0.0" sourceLinked="1"/>
@@ -894,6 +896,7 @@
     </c:plotArea>
     <c:legend>
       <c:legendPos val="r"/>
+      <c:layout/>
       <c:overlay val="0"/>
     </c:legend>
     <c:plotVisOnly val="1"/>
@@ -925,11 +928,13 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
+              <a:rPr lang="en-US"/>
               <a:t>Curva de Calibración Caudalímetro YF-S401 (Frecuencia vs Caudal)</a:t>
             </a:r>
           </a:p>
         </c:rich>
       </c:tx>
+      <c:layout/>
       <c:overlay val="1"/>
     </c:title>
     <c:autoTitleDeleted val="0"/>
@@ -967,6 +972,34 @@
           <c:xVal>
             <c:numRef>
               <c:f>'Ensayo 3 - Caudal Alimentacion'!$G$12:$G$19</c:f>
+              <c:numCache>
+                <c:formatCode>0.000</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>0.28000000000000003</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.43</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.59699999999999998</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.72</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.82</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.91500000000000004</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.96</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1.08</c:v>
+                </c:pt>
+              </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
@@ -975,6 +1008,30 @@
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>60</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>100</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>130</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>150</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>160</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>180</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>190</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>200</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -1014,13 +1071,16 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
+                  <a:rPr lang="en-US"/>
                   <a:t>Caudal Medido Q (L/min)</a:t>
                 </a:r>
               </a:p>
             </c:rich>
           </c:tx>
+          <c:layout/>
           <c:overlay val="1"/>
         </c:title>
+        <c:numFmt formatCode="0.000" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -1046,11 +1106,13 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
+                  <a:rPr lang="en-US"/>
                   <a:t>Frecuencia Generada F (Hz)</a:t>
                 </a:r>
               </a:p>
             </c:rich>
           </c:tx>
+          <c:layout/>
           <c:overlay val="1"/>
         </c:title>
         <c:numFmt formatCode="0.00" sourceLinked="1"/>
@@ -1064,6 +1126,7 @@
     </c:plotArea>
     <c:legend>
       <c:legendPos val="r"/>
+      <c:layout/>
       <c:overlay val="0"/>
     </c:legend>
     <c:plotVisOnly val="1"/>
@@ -1434,13 +1497,13 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:J32"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
-    <col min="3" max="3" width="13" customWidth="1"/>
+    <col min="3" max="3" width="21.140625" customWidth="1"/>
     <col min="4" max="4" width="14" customWidth="1"/>
     <col min="5" max="5" width="15" customWidth="1"/>
     <col min="6" max="7" width="14" customWidth="1"/>
@@ -1448,143 +1511,143 @@
     <col min="10" max="10" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A1" s="28" t="s">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A1" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
-      <c r="G1" s="25"/>
-      <c r="H1" s="25"/>
-      <c r="I1" s="25"/>
-      <c r="J1" s="25"/>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A2" s="36" t="s">
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
+      <c r="I1" s="20"/>
+      <c r="J1" s="20"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A2" s="26" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25"/>
-      <c r="F2" s="25"/>
-      <c r="G2" s="25"/>
-      <c r="H2" s="25"/>
-      <c r="I2" s="25"/>
-      <c r="J2" s="25"/>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A3" s="35" t="s">
+      <c r="B2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
+      <c r="I2" s="20"/>
+      <c r="J2" s="20"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3" s="25" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="25"/>
-      <c r="C3" s="25"/>
-      <c r="D3" s="25"/>
-      <c r="E3" s="25"/>
-      <c r="F3" s="25"/>
-      <c r="G3" s="25"/>
-      <c r="H3" s="25"/>
-      <c r="I3" s="25"/>
-      <c r="J3" s="25"/>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="B3" s="20"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
+      <c r="E3" s="20"/>
+      <c r="F3" s="20"/>
+      <c r="G3" s="20"/>
+      <c r="H3" s="20"/>
+      <c r="I3" s="20"/>
+      <c r="J3" s="20"/>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="24" t="s">
+      <c r="B5" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="25"/>
-      <c r="D5" s="25"/>
+      <c r="C5" s="20"/>
+      <c r="D5" s="20"/>
       <c r="E5" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="F5" s="24" t="s">
+      <c r="F5" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="G5" s="25"/>
-      <c r="H5" s="25"/>
-      <c r="I5" s="25"/>
-      <c r="J5" s="25"/>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="G5" s="20"/>
+      <c r="H5" s="20"/>
+      <c r="I5" s="20"/>
+      <c r="J5" s="20"/>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="24" t="s">
+      <c r="B6" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="25"/>
-      <c r="D6" s="25"/>
+      <c r="C6" s="20"/>
+      <c r="D6" s="20"/>
       <c r="E6" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="F6" s="24" t="s">
+      <c r="F6" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="G6" s="25"/>
-      <c r="H6" s="25"/>
-      <c r="I6" s="25"/>
-      <c r="J6" s="25"/>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="G6" s="20"/>
+      <c r="H6" s="20"/>
+      <c r="I6" s="20"/>
+      <c r="J6" s="20"/>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="24" t="s">
+      <c r="B7" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="25"/>
-      <c r="D7" s="25"/>
+      <c r="C7" s="20"/>
+      <c r="D7" s="20"/>
       <c r="E7" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="F7" s="24" t="s">
+      <c r="F7" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="G7" s="25"/>
-      <c r="H7" s="25"/>
-      <c r="I7" s="25"/>
-      <c r="J7" s="25"/>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="G7" s="20"/>
+      <c r="H7" s="20"/>
+      <c r="I7" s="20"/>
+      <c r="J7" s="20"/>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="24" t="s">
+      <c r="B8" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="C8" s="25"/>
-      <c r="D8" s="25"/>
+      <c r="C8" s="20"/>
+      <c r="D8" s="20"/>
       <c r="E8" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F8" s="24" t="s">
+      <c r="F8" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="G8" s="25"/>
-      <c r="H8" s="25"/>
-      <c r="I8" s="25"/>
-      <c r="J8" s="25"/>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A9" s="27" t="s">
+      <c r="G8" s="20"/>
+      <c r="H8" s="20"/>
+      <c r="I8" s="20"/>
+      <c r="J8" s="20"/>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" s="31" t="s">
         <v>19</v>
       </c>
-      <c r="B9" s="25"/>
-      <c r="C9" s="25"/>
-      <c r="D9" s="25"/>
-      <c r="E9" s="25"/>
-      <c r="F9" s="25"/>
-      <c r="G9" s="25"/>
-      <c r="H9" s="25"/>
-      <c r="I9" s="25"/>
-      <c r="J9" s="25"/>
-    </row>
-    <row r="11" spans="1:10" ht="26" x14ac:dyDescent="0.35">
+      <c r="B9" s="20"/>
+      <c r="C9" s="20"/>
+      <c r="D9" s="20"/>
+      <c r="E9" s="20"/>
+      <c r="F9" s="20"/>
+      <c r="G9" s="20"/>
+      <c r="H9" s="20"/>
+      <c r="I9" s="20"/>
+      <c r="J9" s="20"/>
+    </row>
+    <row r="11" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>20</v>
       </c>
@@ -1616,297 +1679,329 @@
         <v>29</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="3">
         <v>1</v>
       </c>
       <c r="B12" s="4">
         <v>20</v>
       </c>
-      <c r="C12" s="5"/>
-      <c r="D12" s="6"/>
-      <c r="E12" s="7" t="str">
+      <c r="C12" s="5">
+        <v>1</v>
+      </c>
+      <c r="D12" s="6">
+        <v>280</v>
+      </c>
+      <c r="E12" s="7">
         <f t="shared" ref="E12:E19" si="0">IF(OR(D12="",C12=""),"",D12/C12)</f>
-        <v/>
-      </c>
-      <c r="F12" s="8" t="str">
+        <v>280</v>
+      </c>
+      <c r="F12" s="8">
         <f t="shared" ref="F12:F19" si="1">IF(E12="","",E12/1000)</f>
-        <v/>
-      </c>
-      <c r="G12" s="9" t="str">
+        <v>0.28000000000000003</v>
+      </c>
+      <c r="G12" s="9">
         <f t="shared" ref="G12:G19" si="2">IF(OR(B12="",E12=""),"",E12/B12)</f>
-        <v/>
+        <v>14</v>
       </c>
       <c r="H12" s="7">
-        <f t="shared" ref="H12:H19" si="3">IF(B12="","",B12*13.6)</f>
+        <f>IF(B12="","",B12*13.6)</f>
         <v>272</v>
       </c>
-      <c r="I12" s="10" t="str">
-        <f t="shared" ref="I12:I19" si="4">IF(OR(G12="",E12=""),"",((G12-13.6)/13.6)*100)</f>
-        <v/>
+      <c r="I12" s="10">
+        <f t="shared" ref="I12:I19" si="3">IF(OR(G12="",E12=""),"",((G12-13.6)/13.6)*100)</f>
+        <v>2.9411764705882382</v>
       </c>
       <c r="J12" s="11" t="str">
-        <f t="shared" ref="J12:J19" si="5">IF(E12="","-",IF(ABS(I12)&lt;=10,"OK","REVISAR"))</f>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+        <f t="shared" ref="J12:J19" si="4">IF(E12="","-",IF(ABS(I12)&lt;=10,"OK","REVISAR"))</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="3">
         <v>2</v>
       </c>
       <c r="B13" s="4">
         <v>30</v>
       </c>
-      <c r="C13" s="5"/>
-      <c r="D13" s="6"/>
-      <c r="E13" s="7" t="str">
+      <c r="C13" s="5">
+        <v>1</v>
+      </c>
+      <c r="D13" s="6">
+        <v>430</v>
+      </c>
+      <c r="E13" s="7">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="F13" s="8" t="str">
+        <v>430</v>
+      </c>
+      <c r="F13" s="8">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="G13" s="9" t="str">
+        <v>0.43</v>
+      </c>
+      <c r="G13" s="9">
         <f t="shared" si="2"/>
-        <v/>
+        <v>14.333333333333334</v>
       </c>
       <c r="H13" s="7">
+        <f t="shared" ref="H12:H19" si="5">IF(B13="","",B13*13.6)</f>
+        <v>408</v>
+      </c>
+      <c r="I13" s="10">
         <f t="shared" si="3"/>
-        <v>408</v>
-      </c>
-      <c r="I13" s="10" t="str">
+        <v>5.3921568627451055</v>
+      </c>
+      <c r="J13" s="11" t="str">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="J13" s="11" t="str">
-        <f t="shared" si="5"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="3">
         <v>3</v>
       </c>
       <c r="B14" s="4">
         <v>40</v>
       </c>
-      <c r="C14" s="5"/>
-      <c r="D14" s="6"/>
-      <c r="E14" s="7" t="str">
+      <c r="C14" s="5">
+        <v>1</v>
+      </c>
+      <c r="D14" s="6">
+        <v>597</v>
+      </c>
+      <c r="E14" s="7">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="F14" s="8" t="str">
+        <v>597</v>
+      </c>
+      <c r="F14" s="8">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="G14" s="9" t="str">
+        <v>0.59699999999999998</v>
+      </c>
+      <c r="G14" s="9">
         <f t="shared" si="2"/>
-        <v/>
+        <v>14.925000000000001</v>
       </c>
       <c r="H14" s="7">
+        <f t="shared" si="5"/>
+        <v>544</v>
+      </c>
+      <c r="I14" s="10">
         <f t="shared" si="3"/>
-        <v>544</v>
-      </c>
-      <c r="I14" s="10" t="str">
+        <v>9.7426470588235379</v>
+      </c>
+      <c r="J14" s="11" t="str">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="J14" s="11" t="str">
-        <f t="shared" si="5"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="3">
         <v>4</v>
       </c>
       <c r="B15" s="4">
         <v>50</v>
       </c>
-      <c r="C15" s="5"/>
-      <c r="D15" s="6"/>
-      <c r="E15" s="7" t="str">
+      <c r="C15" s="5">
+        <v>1</v>
+      </c>
+      <c r="D15" s="6">
+        <v>720</v>
+      </c>
+      <c r="E15" s="7">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="F15" s="8" t="str">
+        <v>720</v>
+      </c>
+      <c r="F15" s="8">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="G15" s="9" t="str">
+        <v>0.72</v>
+      </c>
+      <c r="G15" s="9">
         <f t="shared" si="2"/>
-        <v/>
+        <v>14.4</v>
       </c>
       <c r="H15" s="7">
+        <f t="shared" si="5"/>
+        <v>680</v>
+      </c>
+      <c r="I15" s="10">
         <f t="shared" si="3"/>
-        <v>680</v>
-      </c>
-      <c r="I15" s="10" t="str">
+        <v>5.8823529411764763</v>
+      </c>
+      <c r="J15" s="11" t="str">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="J15" s="11" t="str">
-        <f t="shared" si="5"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="3">
         <v>5</v>
       </c>
       <c r="B16" s="4">
         <v>60</v>
       </c>
-      <c r="C16" s="5"/>
-      <c r="D16" s="6"/>
-      <c r="E16" s="7" t="str">
+      <c r="C16" s="5">
+        <v>1</v>
+      </c>
+      <c r="D16" s="6">
+        <v>820</v>
+      </c>
+      <c r="E16" s="7">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="F16" s="8" t="str">
+        <v>820</v>
+      </c>
+      <c r="F16" s="8">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="G16" s="9" t="str">
+        <v>0.82</v>
+      </c>
+      <c r="G16" s="9">
         <f t="shared" si="2"/>
-        <v/>
+        <v>13.666666666666666</v>
       </c>
       <c r="H16" s="7">
+        <f t="shared" si="5"/>
+        <v>816</v>
+      </c>
+      <c r="I16" s="10">
         <f t="shared" si="3"/>
-        <v>816</v>
-      </c>
-      <c r="I16" s="10" t="str">
+        <v>0.49019607843137081</v>
+      </c>
+      <c r="J16" s="11" t="str">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="J16" s="11" t="str">
-        <f t="shared" si="5"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="3">
         <v>6</v>
       </c>
       <c r="B17" s="4">
         <v>70</v>
       </c>
-      <c r="C17" s="5"/>
-      <c r="D17" s="6"/>
-      <c r="E17" s="7" t="str">
+      <c r="C17" s="5">
+        <v>1</v>
+      </c>
+      <c r="D17" s="6">
+        <v>915</v>
+      </c>
+      <c r="E17" s="7">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="F17" s="8" t="str">
+        <v>915</v>
+      </c>
+      <c r="F17" s="8">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="G17" s="9" t="str">
+        <v>0.91500000000000004</v>
+      </c>
+      <c r="G17" s="9">
         <f t="shared" si="2"/>
-        <v/>
+        <v>13.071428571428571</v>
       </c>
       <c r="H17" s="7">
+        <f t="shared" si="5"/>
+        <v>952</v>
+      </c>
+      <c r="I17" s="10">
         <f t="shared" si="3"/>
-        <v>952</v>
-      </c>
-      <c r="I17" s="10" t="str">
+        <v>-3.886554621848739</v>
+      </c>
+      <c r="J17" s="11" t="str">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="J17" s="11" t="str">
-        <f t="shared" si="5"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="3">
         <v>7</v>
       </c>
       <c r="B18" s="4">
         <v>80</v>
       </c>
-      <c r="C18" s="5"/>
-      <c r="D18" s="6"/>
-      <c r="E18" s="7" t="str">
+      <c r="C18" s="5">
+        <v>0.5</v>
+      </c>
+      <c r="D18" s="6">
+        <v>480</v>
+      </c>
+      <c r="E18" s="7">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="F18" s="8" t="str">
+        <v>960</v>
+      </c>
+      <c r="F18" s="8">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="G18" s="9" t="str">
+        <v>0.96</v>
+      </c>
+      <c r="G18" s="9">
         <f t="shared" si="2"/>
-        <v/>
+        <v>12</v>
       </c>
       <c r="H18" s="7">
+        <f t="shared" si="5"/>
+        <v>1088</v>
+      </c>
+      <c r="I18" s="10">
         <f t="shared" si="3"/>
-        <v>1088</v>
-      </c>
-      <c r="I18" s="10" t="str">
+        <v>-11.764705882352938</v>
+      </c>
+      <c r="J18" s="11" t="str">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="J18" s="11" t="str">
-        <f t="shared" si="5"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
+        <v>REVISAR</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" s="3">
         <v>8</v>
       </c>
       <c r="B19" s="4">
         <v>90</v>
       </c>
-      <c r="C19" s="5"/>
-      <c r="D19" s="6"/>
-      <c r="E19" s="7" t="str">
+      <c r="C19" s="5">
+        <v>0.5</v>
+      </c>
+      <c r="D19" s="6">
+        <v>540</v>
+      </c>
+      <c r="E19" s="7">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="F19" s="8" t="str">
+        <v>1080</v>
+      </c>
+      <c r="F19" s="8">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="G19" s="9" t="str">
+        <v>1.08</v>
+      </c>
+      <c r="G19" s="9">
         <f t="shared" si="2"/>
-        <v/>
+        <v>12</v>
       </c>
       <c r="H19" s="7">
+        <f t="shared" si="5"/>
+        <v>1224</v>
+      </c>
+      <c r="I19" s="10">
         <f t="shared" si="3"/>
-        <v>1224</v>
-      </c>
-      <c r="I19" s="10" t="str">
+        <v>-11.764705882352938</v>
+      </c>
+      <c r="J19" s="11" t="str">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="J19" s="11" t="str">
-        <f t="shared" si="5"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A21" s="34" t="s">
+        <v>REVISAR</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A21" s="24" t="s">
         <v>30</v>
       </c>
-      <c r="B21" s="25"/>
-      <c r="C21" s="25"/>
-      <c r="D21" s="25"/>
-      <c r="E21" s="25"/>
-      <c r="F21" s="25"/>
-      <c r="G21" s="25"/>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A22" s="22" t="s">
+      <c r="B21" s="20"/>
+      <c r="C21" s="20"/>
+      <c r="D21" s="20"/>
+      <c r="E21" s="20"/>
+      <c r="F21" s="20"/>
+      <c r="G21" s="20"/>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A22" s="21" t="s">
         <v>31</v>
       </c>
-      <c r="B22" s="23"/>
-      <c r="C22" s="13" t="e">
+      <c r="B22" s="22"/>
+      <c r="C22" s="13">
         <f>AVERAGE(G12:G19)</f>
-        <v>#DIV/0!</v>
+        <v>13.549553571428572</v>
       </c>
       <c r="D22" s="14" t="s">
         <v>32</v>
@@ -1915,11 +2010,11 @@
       <c r="F22" s="12"/>
       <c r="G22" s="12"/>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A23" s="22" t="s">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A23" s="21" t="s">
         <v>33</v>
       </c>
-      <c r="B23" s="23"/>
+      <c r="B23" s="22"/>
       <c r="C23" s="13" t="e">
         <f ca="1">_xludf.STDEV.S(G12:G19)</f>
         <v>#NAME?</v>
@@ -1931,11 +2026,11 @@
       <c r="F23" s="12"/>
       <c r="G23" s="12"/>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A24" s="22" t="s">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A24" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="B24" s="23"/>
+      <c r="B24" s="22"/>
       <c r="C24" s="15" t="e">
         <f ca="1">(C23/C22)*100</f>
         <v>#NAME?</v>
@@ -1947,14 +2042,14 @@
       <c r="F24" s="12"/>
       <c r="G24" s="12"/>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A25" s="22" t="s">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A25" s="21" t="s">
         <v>36</v>
       </c>
-      <c r="B25" s="23"/>
-      <c r="C25" s="13" t="e">
+      <c r="B25" s="22"/>
+      <c r="C25" s="13">
         <f>SLOPE(E12:E19,B12:B19)</f>
-        <v>#DIV/0!</v>
+        <v>11.076190476190476</v>
       </c>
       <c r="D25" s="14" t="s">
         <v>32</v>
@@ -1963,14 +2058,14 @@
       <c r="F25" s="12"/>
       <c r="G25" s="12"/>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A26" s="22" t="s">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A26" s="21" t="s">
         <v>37</v>
       </c>
-      <c r="B26" s="23"/>
-      <c r="C26" s="15" t="e">
+      <c r="B26" s="22"/>
+      <c r="C26" s="15">
         <f>INTERCEPT(E12:E19,B12:B19)</f>
-        <v>#DIV/0!</v>
+        <v>116.05952380952385</v>
       </c>
       <c r="D26" s="14" t="s">
         <v>38</v>
@@ -1979,14 +2074,14 @@
       <c r="F26" s="12"/>
       <c r="G26" s="12"/>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A27" s="22" t="s">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A27" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="B27" s="23"/>
-      <c r="C27" s="13" t="e">
+      <c r="B27" s="22"/>
+      <c r="C27" s="13">
         <f>RSQ(E12:E19,B12:B19)</f>
-        <v>#DIV/0!</v>
+        <v>0.976187341183121</v>
       </c>
       <c r="D27" s="14" t="s">
         <v>40</v>
@@ -1995,53 +2090,63 @@
       <c r="F27" s="12"/>
       <c r="G27" s="12"/>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A29" s="26" t="s">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A29" s="30" t="s">
         <v>41</v>
       </c>
-      <c r="B29" s="20"/>
-      <c r="C29" s="20"/>
-      <c r="D29" s="20"/>
-      <c r="E29" s="20"/>
-      <c r="F29" s="20"/>
-      <c r="G29" s="21"/>
-    </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A30" s="26" t="s">
+      <c r="B29" s="28"/>
+      <c r="C29" s="28"/>
+      <c r="D29" s="28"/>
+      <c r="E29" s="28"/>
+      <c r="F29" s="28"/>
+      <c r="G29" s="29"/>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A30" s="30" t="s">
         <v>42</v>
       </c>
-      <c r="B30" s="29"/>
-      <c r="C30" s="29"/>
-      <c r="D30" s="29"/>
-      <c r="E30" s="30"/>
-      <c r="F30" s="37" t="e">
+      <c r="B30" s="32"/>
+      <c r="C30" s="32"/>
+      <c r="D30" s="32"/>
+      <c r="E30" s="33"/>
+      <c r="F30" s="37">
         <f>C25</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G30" s="30"/>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A31" s="31"/>
-      <c r="B31" s="32"/>
-      <c r="C31" s="32"/>
-      <c r="D31" s="32"/>
-      <c r="E31" s="33"/>
-      <c r="F31" s="31"/>
-      <c r="G31" s="33"/>
-    </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A32" s="19" t="s">
+        <v>11.076190476190476</v>
+      </c>
+      <c r="G30" s="33"/>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A31" s="34"/>
+      <c r="B31" s="35"/>
+      <c r="C31" s="35"/>
+      <c r="D31" s="35"/>
+      <c r="E31" s="36"/>
+      <c r="F31" s="34"/>
+      <c r="G31" s="36"/>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A32" s="27" t="s">
         <v>43</v>
       </c>
-      <c r="B32" s="20"/>
-      <c r="C32" s="20"/>
-      <c r="D32" s="20"/>
-      <c r="E32" s="20"/>
-      <c r="F32" s="20"/>
-      <c r="G32" s="21"/>
+      <c r="B32" s="28"/>
+      <c r="C32" s="28"/>
+      <c r="D32" s="28"/>
+      <c r="E32" s="28"/>
+      <c r="F32" s="28"/>
+      <c r="G32" s="29"/>
     </row>
   </sheetData>
   <mergeCells count="23">
+    <mergeCell ref="A32:G32"/>
+    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="A29:G29"/>
+    <mergeCell ref="F6:J6"/>
+    <mergeCell ref="F7:J7"/>
+    <mergeCell ref="A25:B25"/>
+    <mergeCell ref="A9:J9"/>
+    <mergeCell ref="A30:E31"/>
+    <mergeCell ref="F30:G31"/>
     <mergeCell ref="F5:J5"/>
     <mergeCell ref="A27:B27"/>
     <mergeCell ref="B6:D6"/>
@@ -2055,16 +2160,6 @@
     <mergeCell ref="A21:G21"/>
     <mergeCell ref="A3:J3"/>
     <mergeCell ref="A2:J2"/>
-    <mergeCell ref="A32:G32"/>
-    <mergeCell ref="A24:B24"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="A29:G29"/>
-    <mergeCell ref="F6:J6"/>
-    <mergeCell ref="F7:J7"/>
-    <mergeCell ref="A25:B25"/>
-    <mergeCell ref="A9:J9"/>
-    <mergeCell ref="A30:E31"/>
-    <mergeCell ref="F30:G31"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing r:id="rId1"/>
@@ -2072,9 +2167,9 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:L33"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="13" customWidth="1"/>
@@ -2090,159 +2185,159 @@
     <col min="12" max="12" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A1" s="28" t="s">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
-      <c r="G1" s="25"/>
-      <c r="H1" s="25"/>
-      <c r="I1" s="25"/>
-      <c r="J1" s="25"/>
-      <c r="K1" s="25"/>
-      <c r="L1" s="25"/>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A2" s="36" t="s">
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
+      <c r="I1" s="20"/>
+      <c r="J1" s="20"/>
+      <c r="K1" s="20"/>
+      <c r="L1" s="20"/>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A2" s="26" t="s">
         <v>44</v>
       </c>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25"/>
-      <c r="F2" s="25"/>
-      <c r="G2" s="25"/>
-      <c r="H2" s="25"/>
-      <c r="I2" s="25"/>
-      <c r="J2" s="25"/>
-      <c r="K2" s="25"/>
-      <c r="L2" s="25"/>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A3" s="35" t="s">
+      <c r="B2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
+      <c r="I2" s="20"/>
+      <c r="J2" s="20"/>
+      <c r="K2" s="20"/>
+      <c r="L2" s="20"/>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A3" s="25" t="s">
         <v>45</v>
       </c>
-      <c r="B3" s="25"/>
-      <c r="C3" s="25"/>
-      <c r="D3" s="25"/>
-      <c r="E3" s="25"/>
-      <c r="F3" s="25"/>
-      <c r="G3" s="25"/>
-      <c r="H3" s="25"/>
-      <c r="I3" s="25"/>
-      <c r="J3" s="25"/>
-      <c r="K3" s="25"/>
-      <c r="L3" s="25"/>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="B3" s="20"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
+      <c r="E3" s="20"/>
+      <c r="F3" s="20"/>
+      <c r="G3" s="20"/>
+      <c r="H3" s="20"/>
+      <c r="I3" s="20"/>
+      <c r="J3" s="20"/>
+      <c r="K3" s="20"/>
+      <c r="L3" s="20"/>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B5" s="24" t="s">
+      <c r="B5" s="19" t="s">
         <v>47</v>
       </c>
-      <c r="C5" s="25"/>
-      <c r="D5" s="25"/>
-      <c r="E5" s="25"/>
+      <c r="C5" s="20"/>
+      <c r="D5" s="20"/>
+      <c r="E5" s="20"/>
       <c r="F5" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="G5" s="24" t="s">
+      <c r="G5" s="19" t="s">
         <v>49</v>
       </c>
-      <c r="H5" s="25"/>
-      <c r="I5" s="25"/>
-      <c r="J5" s="25"/>
-      <c r="K5" s="25"/>
-      <c r="L5" s="25"/>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="H5" s="20"/>
+      <c r="I5" s="20"/>
+      <c r="J5" s="20"/>
+      <c r="K5" s="20"/>
+      <c r="L5" s="20"/>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="B6" s="24" t="s">
+      <c r="B6" s="19" t="s">
         <v>51</v>
       </c>
-      <c r="C6" s="25"/>
-      <c r="D6" s="25"/>
-      <c r="E6" s="25"/>
+      <c r="C6" s="20"/>
+      <c r="D6" s="20"/>
+      <c r="E6" s="20"/>
       <c r="F6" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="G6" s="24" t="s">
+      <c r="G6" s="19" t="s">
         <v>53</v>
       </c>
-      <c r="H6" s="25"/>
-      <c r="I6" s="25"/>
-      <c r="J6" s="25"/>
-      <c r="K6" s="25"/>
-      <c r="L6" s="25"/>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="H6" s="20"/>
+      <c r="I6" s="20"/>
+      <c r="J6" s="20"/>
+      <c r="K6" s="20"/>
+      <c r="L6" s="20"/>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="B7" s="24" t="s">
+      <c r="B7" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="C7" s="25"/>
-      <c r="D7" s="25"/>
-      <c r="E7" s="25"/>
+      <c r="C7" s="20"/>
+      <c r="D7" s="20"/>
+      <c r="E7" s="20"/>
       <c r="F7" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="G7" s="24" t="s">
+      <c r="G7" s="19" t="s">
         <v>57</v>
       </c>
-      <c r="H7" s="25"/>
-      <c r="I7" s="25"/>
-      <c r="J7" s="25"/>
-      <c r="K7" s="25"/>
-      <c r="L7" s="25"/>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="H7" s="20"/>
+      <c r="I7" s="20"/>
+      <c r="J7" s="20"/>
+      <c r="K7" s="20"/>
+      <c r="L7" s="20"/>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="24" t="s">
+      <c r="B8" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="C8" s="25"/>
-      <c r="D8" s="25"/>
-      <c r="E8" s="25"/>
+      <c r="C8" s="20"/>
+      <c r="D8" s="20"/>
+      <c r="E8" s="20"/>
       <c r="F8" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="G8" s="24" t="s">
+      <c r="G8" s="19" t="s">
         <v>59</v>
       </c>
-      <c r="H8" s="25"/>
-      <c r="I8" s="25"/>
-      <c r="J8" s="25"/>
-      <c r="K8" s="25"/>
-      <c r="L8" s="25"/>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A9" s="27" t="s">
+      <c r="H8" s="20"/>
+      <c r="I8" s="20"/>
+      <c r="J8" s="20"/>
+      <c r="K8" s="20"/>
+      <c r="L8" s="20"/>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A9" s="31" t="s">
         <v>60</v>
       </c>
-      <c r="B9" s="25"/>
-      <c r="C9" s="25"/>
-      <c r="D9" s="25"/>
-      <c r="E9" s="25"/>
-      <c r="F9" s="25"/>
-      <c r="G9" s="25"/>
-      <c r="H9" s="25"/>
-      <c r="I9" s="25"/>
-      <c r="J9" s="25"/>
-      <c r="K9" s="25"/>
-      <c r="L9" s="25"/>
-    </row>
-    <row r="11" spans="1:12" ht="26" x14ac:dyDescent="0.35">
+      <c r="B9" s="20"/>
+      <c r="C9" s="20"/>
+      <c r="D9" s="20"/>
+      <c r="E9" s="20"/>
+      <c r="F9" s="20"/>
+      <c r="G9" s="20"/>
+      <c r="H9" s="20"/>
+      <c r="I9" s="20"/>
+      <c r="J9" s="20"/>
+      <c r="K9" s="20"/>
+      <c r="L9" s="20"/>
+    </row>
+    <row r="11" spans="1:12" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>20</v>
       </c>
@@ -2280,337 +2375,385 @@
         <v>66</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" s="3">
         <v>1</v>
       </c>
       <c r="B12" s="4">
         <v>20</v>
       </c>
-      <c r="C12" s="16"/>
-      <c r="D12" s="5"/>
-      <c r="E12" s="6"/>
-      <c r="F12" s="7" t="str">
+      <c r="C12" s="16">
+        <v>60</v>
+      </c>
+      <c r="D12" s="5">
+        <v>1</v>
+      </c>
+      <c r="E12" s="6">
+        <v>280</v>
+      </c>
+      <c r="F12" s="7">
         <f t="shared" ref="F12:F19" si="0">IF(OR(E12="",D12=""),"",E12/D12)</f>
-        <v/>
-      </c>
-      <c r="G12" s="8" t="str">
+        <v>280</v>
+      </c>
+      <c r="G12" s="8">
         <f t="shared" ref="G12:G19" si="1">IF(F12="","",F12/1000)</f>
-        <v/>
-      </c>
-      <c r="H12" s="17" t="str">
+        <v>0.28000000000000003</v>
+      </c>
+      <c r="H12" s="17">
         <f t="shared" ref="H12:H19" si="2">IF(OR(C12="",G12=""),"",C12/G12)</f>
-        <v/>
-      </c>
-      <c r="I12" s="7" t="str">
+        <v>214.28571428571428</v>
+      </c>
+      <c r="I12" s="7">
         <f t="shared" ref="I12:I19" si="3">IF(H12="","",H12*60)</f>
-        <v/>
-      </c>
-      <c r="J12" s="7" t="str">
+        <v>12857.142857142857</v>
+      </c>
+      <c r="J12" s="7">
         <f t="shared" ref="J12:J19" si="4">IF(C12="","",(C12*1000)/154.62)</f>
-        <v/>
-      </c>
-      <c r="K12" s="10" t="str">
+        <v>388.04811796662784</v>
+      </c>
+      <c r="K12" s="10">
         <f t="shared" ref="K12:K19" si="5">IF(OR(F12="",J12=""),"",((J12-F12)/F12)*100)</f>
-        <v/>
+        <v>38.588613559509945</v>
       </c>
       <c r="L12" s="11" t="str">
         <f t="shared" ref="L12:L19" si="6">IF(F12="","-",IF(ABS(K12)&lt;=5,"EXCELENTE",IF(ABS(K12)&lt;=12,"BUENA","DESVIADA")))</f>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
+        <v>DESVIADA</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" s="3">
         <v>2</v>
       </c>
       <c r="B13" s="4">
         <v>30</v>
       </c>
-      <c r="C13" s="16"/>
-      <c r="D13" s="5"/>
-      <c r="E13" s="6"/>
-      <c r="F13" s="7" t="str">
+      <c r="C13" s="16">
+        <v>100</v>
+      </c>
+      <c r="D13" s="5">
+        <v>1</v>
+      </c>
+      <c r="E13" s="6">
+        <v>430</v>
+      </c>
+      <c r="F13" s="7">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G13" s="8" t="str">
+        <v>430</v>
+      </c>
+      <c r="G13" s="8">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="H13" s="17" t="str">
+        <v>0.43</v>
+      </c>
+      <c r="H13" s="17">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="I13" s="7" t="str">
+        <v>232.55813953488374</v>
+      </c>
+      <c r="I13" s="7">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="J13" s="7" t="str">
+        <v>13953.488372093025</v>
+      </c>
+      <c r="J13" s="7">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="K13" s="10" t="str">
+        <v>646.74686327771303</v>
+      </c>
+      <c r="K13" s="10">
         <f t="shared" si="5"/>
-        <v/>
+        <v>50.406247273886748</v>
       </c>
       <c r="L13" s="11" t="str">
         <f t="shared" si="6"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.35">
+        <v>DESVIADA</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" s="3">
         <v>3</v>
       </c>
       <c r="B14" s="4">
         <v>40</v>
       </c>
-      <c r="C14" s="16"/>
-      <c r="D14" s="5"/>
-      <c r="E14" s="6"/>
-      <c r="F14" s="7" t="str">
+      <c r="C14" s="16">
+        <v>130</v>
+      </c>
+      <c r="D14" s="5">
+        <v>1</v>
+      </c>
+      <c r="E14" s="6">
+        <v>597</v>
+      </c>
+      <c r="F14" s="7">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G14" s="8" t="str">
+        <v>597</v>
+      </c>
+      <c r="G14" s="8">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="H14" s="17" t="str">
+        <v>0.59699999999999998</v>
+      </c>
+      <c r="H14" s="17">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="I14" s="7" t="str">
+        <v>217.75544388609717</v>
+      </c>
+      <c r="I14" s="7">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="J14" s="7" t="str">
+        <v>13065.326633165831</v>
+      </c>
+      <c r="J14" s="7">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="K14" s="10" t="str">
+        <v>840.77092226102695</v>
+      </c>
+      <c r="K14" s="10">
         <f t="shared" si="5"/>
-        <v/>
+        <v>40.832650294979388</v>
       </c>
       <c r="L14" s="11" t="str">
         <f t="shared" si="6"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
+        <v>DESVIADA</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" s="3">
         <v>4</v>
       </c>
       <c r="B15" s="4">
         <v>50</v>
       </c>
-      <c r="C15" s="16"/>
-      <c r="D15" s="5"/>
-      <c r="E15" s="6"/>
-      <c r="F15" s="7" t="str">
+      <c r="C15" s="16">
+        <v>150</v>
+      </c>
+      <c r="D15" s="5">
+        <v>1</v>
+      </c>
+      <c r="E15" s="6">
+        <v>720</v>
+      </c>
+      <c r="F15" s="7">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G15" s="8" t="str">
+        <v>720</v>
+      </c>
+      <c r="G15" s="8">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="H15" s="17" t="str">
+        <v>0.72</v>
+      </c>
+      <c r="H15" s="17">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="I15" s="7" t="str">
+        <v>208.33333333333334</v>
+      </c>
+      <c r="I15" s="7">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="J15" s="7" t="str">
+        <v>12500</v>
+      </c>
+      <c r="J15" s="7">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="K15" s="10" t="str">
+        <v>970.12029491656961</v>
+      </c>
+      <c r="K15" s="10">
         <f t="shared" si="5"/>
-        <v/>
+        <v>34.738929849523558</v>
       </c>
       <c r="L15" s="11" t="str">
         <f t="shared" si="6"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.35">
+        <v>DESVIADA</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" s="3">
         <v>5</v>
       </c>
       <c r="B16" s="4">
         <v>60</v>
       </c>
-      <c r="C16" s="16"/>
-      <c r="D16" s="5"/>
-      <c r="E16" s="6"/>
-      <c r="F16" s="7" t="str">
+      <c r="C16" s="16">
+        <v>160</v>
+      </c>
+      <c r="D16" s="5">
+        <v>1</v>
+      </c>
+      <c r="E16" s="6">
+        <v>820</v>
+      </c>
+      <c r="F16" s="7">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G16" s="8" t="str">
+        <v>820</v>
+      </c>
+      <c r="G16" s="8">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="H16" s="17" t="str">
+        <v>0.82</v>
+      </c>
+      <c r="H16" s="17">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="I16" s="7" t="str">
+        <v>195.1219512195122</v>
+      </c>
+      <c r="I16" s="7">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="J16" s="7" t="str">
+        <v>11707.317073170732</v>
+      </c>
+      <c r="J16" s="7">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="K16" s="10" t="str">
+        <v>1034.794981244341</v>
+      </c>
+      <c r="K16" s="10">
         <f t="shared" si="5"/>
-        <v/>
+        <v>26.194509907846463</v>
       </c>
       <c r="L16" s="11" t="str">
         <f t="shared" si="6"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.35">
+        <v>DESVIADA</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" s="3">
         <v>6</v>
       </c>
       <c r="B17" s="4">
         <v>70</v>
       </c>
-      <c r="C17" s="16"/>
-      <c r="D17" s="5"/>
-      <c r="E17" s="6"/>
-      <c r="F17" s="7" t="str">
+      <c r="C17" s="16">
+        <v>180</v>
+      </c>
+      <c r="D17" s="5">
+        <v>1</v>
+      </c>
+      <c r="E17" s="6">
+        <v>915</v>
+      </c>
+      <c r="F17" s="7">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G17" s="8" t="str">
+        <v>915</v>
+      </c>
+      <c r="G17" s="8">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="H17" s="17" t="str">
+        <v>0.91500000000000004</v>
+      </c>
+      <c r="H17" s="17">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="I17" s="7" t="str">
+        <v>196.72131147540983</v>
+      </c>
+      <c r="I17" s="7">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="J17" s="7" t="str">
+        <v>11803.27868852459</v>
+      </c>
+      <c r="J17" s="7">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="K17" s="10" t="str">
+        <v>1164.1443538998835</v>
+      </c>
+      <c r="K17" s="10">
         <f t="shared" si="5"/>
-        <v/>
+        <v>27.228891136599291</v>
       </c>
       <c r="L17" s="11" t="str">
         <f t="shared" si="6"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.35">
+        <v>DESVIADA</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18" s="3">
         <v>7</v>
       </c>
       <c r="B18" s="4">
         <v>80</v>
       </c>
-      <c r="C18" s="16"/>
-      <c r="D18" s="5"/>
-      <c r="E18" s="6"/>
-      <c r="F18" s="7" t="str">
+      <c r="C18" s="16">
+        <v>190</v>
+      </c>
+      <c r="D18" s="5">
+        <v>0.5</v>
+      </c>
+      <c r="E18" s="6">
+        <v>480</v>
+      </c>
+      <c r="F18" s="7">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G18" s="8" t="str">
+        <v>960</v>
+      </c>
+      <c r="G18" s="8">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="H18" s="17" t="str">
+        <v>0.96</v>
+      </c>
+      <c r="H18" s="17">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="I18" s="7" t="str">
+        <v>197.91666666666669</v>
+      </c>
+      <c r="I18" s="7">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="J18" s="7" t="str">
+        <v>11875.000000000002</v>
+      </c>
+      <c r="J18" s="7">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="K18" s="10" t="str">
+        <v>1228.8190402276548</v>
+      </c>
+      <c r="K18" s="10">
         <f t="shared" si="5"/>
-        <v/>
+        <v>28.001983357047372</v>
       </c>
       <c r="L18" s="11" t="str">
         <f t="shared" si="6"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.35">
+        <v>DESVIADA</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" s="3">
         <v>8</v>
       </c>
       <c r="B19" s="4">
         <v>90</v>
       </c>
-      <c r="C19" s="16"/>
-      <c r="D19" s="5"/>
-      <c r="E19" s="6"/>
-      <c r="F19" s="7" t="str">
+      <c r="C19" s="16">
+        <v>200</v>
+      </c>
+      <c r="D19" s="5">
+        <v>0.5</v>
+      </c>
+      <c r="E19" s="6">
+        <v>540</v>
+      </c>
+      <c r="F19" s="7">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G19" s="8" t="str">
+        <v>1080</v>
+      </c>
+      <c r="G19" s="8">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="H19" s="17" t="str">
+        <v>1.08</v>
+      </c>
+      <c r="H19" s="17">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="I19" s="7" t="str">
+        <v>185.18518518518516</v>
+      </c>
+      <c r="I19" s="7">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="J19" s="7" t="str">
+        <v>11111.111111111109</v>
+      </c>
+      <c r="J19" s="7">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="K19" s="10" t="str">
+        <v>1293.4937265554261</v>
+      </c>
+      <c r="K19" s="10">
         <f t="shared" si="5"/>
-        <v/>
+        <v>19.767937644020932</v>
       </c>
       <c r="L19" s="11" t="str">
         <f t="shared" si="6"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A21" s="34" t="s">
+        <v>DESVIADA</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A21" s="24" t="s">
         <v>67</v>
       </c>
-      <c r="B21" s="25"/>
-      <c r="C21" s="25"/>
-      <c r="D21" s="25"/>
-      <c r="E21" s="25"/>
-      <c r="F21" s="25"/>
-      <c r="G21" s="25"/>
-    </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A22" s="22" t="s">
+      <c r="B21" s="20"/>
+      <c r="C21" s="20"/>
+      <c r="D21" s="20"/>
+      <c r="E21" s="20"/>
+      <c r="F21" s="20"/>
+      <c r="G21" s="20"/>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A22" s="21" t="s">
         <v>68</v>
       </c>
-      <c r="B22" s="23"/>
-      <c r="C22" s="15" t="e">
+      <c r="B22" s="22"/>
+      <c r="C22" s="15">
         <f>AVERAGE(H12:H19)</f>
-        <v>#DIV/0!</v>
+        <v>205.98471819835035</v>
       </c>
       <c r="D22" s="14" t="s">
         <v>69</v>
@@ -2619,11 +2762,11 @@
       <c r="F22" s="12"/>
       <c r="G22" s="12"/>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A23" s="22" t="s">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A23" s="21" t="s">
         <v>70</v>
       </c>
-      <c r="B23" s="23"/>
+      <c r="B23" s="22"/>
       <c r="C23" s="15" t="e">
         <f ca="1">_xludf.STDEV.S(H12:H19)</f>
         <v>#NAME?</v>
@@ -2635,11 +2778,11 @@
       <c r="F23" s="12"/>
       <c r="G23" s="12"/>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A24" s="22" t="s">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A24" s="21" t="s">
         <v>71</v>
       </c>
-      <c r="B24" s="23"/>
+      <c r="B24" s="22"/>
       <c r="C24" s="15" t="e">
         <f ca="1">(C23/C22)*100</f>
         <v>#NAME?</v>
@@ -2651,14 +2794,14 @@
       <c r="F24" s="12"/>
       <c r="G24" s="12"/>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A25" s="22" t="s">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A25" s="21" t="s">
         <v>72</v>
       </c>
-      <c r="B25" s="23"/>
-      <c r="C25" s="18" t="e">
+      <c r="B25" s="22"/>
+      <c r="C25" s="18">
         <f>AVERAGE(I12:I19)</f>
-        <v>#DIV/0!</v>
+        <v>12359.083091901019</v>
       </c>
       <c r="D25" s="14" t="s">
         <v>73</v>
@@ -2667,14 +2810,14 @@
       <c r="F25" s="12"/>
       <c r="G25" s="12"/>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A26" s="22" t="s">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A26" s="21" t="s">
         <v>74</v>
       </c>
-      <c r="B26" s="23"/>
-      <c r="C26" s="15" t="e">
+      <c r="B26" s="22"/>
+      <c r="C26" s="15">
         <f>SLOPE(C12:C19,G12:G19)</f>
-        <v>#DIV/0!</v>
+        <v>172.72018543726384</v>
       </c>
       <c r="D26" s="14" t="s">
         <v>69</v>
@@ -2683,14 +2826,14 @@
       <c r="F26" s="12"/>
       <c r="G26" s="12"/>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A27" s="22" t="s">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A27" s="21" t="s">
         <v>75</v>
       </c>
-      <c r="B27" s="23"/>
-      <c r="C27" s="15" t="e">
+      <c r="B27" s="22"/>
+      <c r="C27" s="15">
         <f>INTERCEPT(C12:C19,G12:G19)</f>
-        <v>#DIV/0!</v>
+        <v>20.984685511624406</v>
       </c>
       <c r="D27" s="14" t="s">
         <v>76</v>
@@ -2699,14 +2842,14 @@
       <c r="F27" s="12"/>
       <c r="G27" s="12"/>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A28" s="22" t="s">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A28" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="B28" s="23"/>
-      <c r="C28" s="13" t="e">
+      <c r="B28" s="22"/>
+      <c r="C28" s="13">
         <f>RSQ(C12:C19,G12:G19)</f>
-        <v>#DIV/0!</v>
+        <v>0.98492369074913211</v>
       </c>
       <c r="D28" s="14" t="s">
         <v>40</v>
@@ -2715,58 +2858,68 @@
       <c r="F28" s="12"/>
       <c r="G28" s="12"/>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A30" s="26" t="s">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A30" s="30" t="s">
         <v>77</v>
       </c>
-      <c r="B30" s="20"/>
-      <c r="C30" s="20"/>
-      <c r="D30" s="20"/>
-      <c r="E30" s="20"/>
-      <c r="F30" s="20"/>
-      <c r="G30" s="21"/>
-    </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A31" s="39" t="s">
+      <c r="B30" s="28"/>
+      <c r="C30" s="28"/>
+      <c r="D30" s="28"/>
+      <c r="E30" s="28"/>
+      <c r="F30" s="28"/>
+      <c r="G30" s="29"/>
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A31" s="38" t="s">
         <v>78</v>
       </c>
-      <c r="B31" s="20"/>
-      <c r="C31" s="20"/>
-      <c r="D31" s="21"/>
-      <c r="E31" s="38" t="e">
+      <c r="B31" s="28"/>
+      <c r="C31" s="28"/>
+      <c r="D31" s="29"/>
+      <c r="E31" s="40">
         <f>C26</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F31" s="20"/>
-      <c r="G31" s="21"/>
-    </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A32" s="39" t="s">
+        <v>172.72018543726384</v>
+      </c>
+      <c r="F31" s="28"/>
+      <c r="G31" s="29"/>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A32" s="38" t="s">
         <v>79</v>
       </c>
-      <c r="B32" s="20"/>
-      <c r="C32" s="20"/>
-      <c r="D32" s="21"/>
-      <c r="E32" s="40" t="e">
+      <c r="B32" s="28"/>
+      <c r="C32" s="28"/>
+      <c r="D32" s="29"/>
+      <c r="E32" s="39">
         <f>E31*60</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F32" s="20"/>
-      <c r="G32" s="21"/>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A33" s="19" t="s">
+        <v>10363.21112623583</v>
+      </c>
+      <c r="F32" s="28"/>
+      <c r="G32" s="29"/>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A33" s="27" t="s">
         <v>80</v>
       </c>
-      <c r="B33" s="20"/>
-      <c r="C33" s="20"/>
-      <c r="D33" s="20"/>
-      <c r="E33" s="20"/>
-      <c r="F33" s="20"/>
-      <c r="G33" s="21"/>
+      <c r="B33" s="28"/>
+      <c r="C33" s="28"/>
+      <c r="D33" s="28"/>
+      <c r="E33" s="28"/>
+      <c r="F33" s="28"/>
+      <c r="G33" s="29"/>
     </row>
   </sheetData>
   <mergeCells count="26">
+    <mergeCell ref="G6:L6"/>
+    <mergeCell ref="B6:E6"/>
+    <mergeCell ref="E31:G31"/>
+    <mergeCell ref="B5:E5"/>
+    <mergeCell ref="A25:B25"/>
+    <mergeCell ref="B7:E7"/>
+    <mergeCell ref="A30:G30"/>
+    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="B8:E8"/>
+    <mergeCell ref="A24:B24"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A28:B28"/>
     <mergeCell ref="G8:L8"/>
@@ -2783,16 +2936,6 @@
     <mergeCell ref="A2:L2"/>
     <mergeCell ref="A31:D31"/>
     <mergeCell ref="G5:L5"/>
-    <mergeCell ref="A25:B25"/>
-    <mergeCell ref="B7:E7"/>
-    <mergeCell ref="A30:G30"/>
-    <mergeCell ref="A27:B27"/>
-    <mergeCell ref="B8:E8"/>
-    <mergeCell ref="A24:B24"/>
-    <mergeCell ref="G6:L6"/>
-    <mergeCell ref="B6:E6"/>
-    <mergeCell ref="E31:G31"/>
-    <mergeCell ref="B5:E5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing r:id="rId1"/>

</xml_diff>